<commit_message>
Rerun of GO-term analysis
</commit_message>
<xml_diff>
--- a/metadata/dominance_meta_corrected.xlsx
+++ b/metadata/dominance_meta_corrected.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f8cb5b7fcd4c426a/Dokument/Master courses/MASTER THESIS/R project-Master Thesis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebas\Documents\GitHub\Master_thesis_sebastian\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="316" documentId="8_{E6DE9369-E5A4-41F0-AC43-5D1C5DBAA4C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CD10894-756E-49B7-85B0-B5629BF33572}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B76D84-EB72-492E-9713-51A2859741C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FDDCB103-F9DC-4D01-9EF3-13268919B821}"/>
   </bookViews>
@@ -1798,7 +1798,7 @@
     <t xml:space="preserve">Possibly ambigous sex, below -50 in the PCA, strays from the other female samples.  But was kept in my thesis </t>
   </si>
   <si>
-    <t xml:space="preserve">NOTE! I relabeled from Male to Female here. Clustered deep with female samples in PCA. But was noted as Male during sampling/sequencing </t>
+    <t xml:space="preserve">Possible mislabel. This sample clusters deep with female samples in PCA. </t>
   </si>
 </sst>
 </file>
@@ -2535,10 +2535,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" connectionId="1" xr16:uid="{340F2CCC-41FD-4189-886C-C1F594AAE06C}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh nextId="21" unboundColumnsRight="6">
@@ -2569,7 +2565,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E8C6FE40-3448-4493-A6D4-E23E5B03B56E}" name="metadata_for_manual_correction" displayName="metadata_for_manual_correction" ref="A1:Q73" tableType="queryTable" totalsRowShown="0" headerRowDxfId="20" headerRowBorderDxfId="19" tableBorderDxfId="18" totalsRowBorderDxfId="17">
   <autoFilter ref="A1:Q73" xr:uid="{E8C6FE40-3448-4493-A6D4-E23E5B03B56E}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q73">
-    <sortCondition ref="A1:A73"/>
+    <sortCondition ref="K1:K73"/>
   </sortState>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{C06F7C9D-D987-4980-A068-0DCA6F5CF582}" uniqueName="1" name="Run" queryTableFieldId="1" dataDxfId="16"/>
@@ -3139,28 +3135,28 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="B5" s="9">
-        <v>9412089720</v>
+        <v>26660551242</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="H5" s="2">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>307</v>
@@ -3169,100 +3165,100 @@
         <v>308</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>560</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="M5" s="1" t="s">
         <v>573</v>
       </c>
       <c r="N5" s="2">
         <v>1</v>
       </c>
-      <c r="O5" s="11" t="s">
-        <v>363</v>
-      </c>
-      <c r="P5" s="11" t="s">
-        <v>397</v>
+      <c r="O5" s="21" t="s">
+        <v>366</v>
+      </c>
+      <c r="P5" s="21" t="s">
+        <v>400</v>
       </c>
       <c r="Q5" s="19"/>
     </row>
-    <row r="6" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="B6" s="9">
-        <v>9959631122</v>
+        <v>15439369480</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>310</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="I6" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="G6" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="H6" s="2">
+        <v>17</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="K6" s="3" t="s">
-        <v>309</v>
-      </c>
-      <c r="L6" s="3" t="s">
+      <c r="K6" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="L6" s="2" t="s">
         <v>560</v>
       </c>
       <c r="M6" s="1" t="s">
         <v>573</v>
       </c>
-      <c r="N6" s="3">
+      <c r="N6" s="2">
         <v>1</v>
       </c>
-      <c r="O6" s="11" t="s">
-        <v>364</v>
-      </c>
-      <c r="P6" s="11" t="s">
-        <v>398</v>
-      </c>
-      <c r="Q6" s="19"/>
+      <c r="O6" s="21" t="s">
+        <v>367</v>
+      </c>
+      <c r="P6" s="21" t="s">
+        <v>401</v>
+      </c>
+      <c r="Q6" s="20"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="12" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="B7" s="9">
-        <v>12797457172</v>
+        <v>6734916496</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="H7" s="2">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>307</v>
@@ -3271,7 +3267,7 @@
         <v>308</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>560</v>
@@ -3283,2493 +3279,2495 @@
         <v>1</v>
       </c>
       <c r="O7" s="11" t="s">
-        <v>365</v>
-      </c>
-      <c r="P7" s="11" t="s">
-        <v>399</v>
-      </c>
-      <c r="Q7" s="19"/>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+        <v>368</v>
+      </c>
+      <c r="P7" s="21" t="s">
+        <v>402</v>
+      </c>
+      <c r="Q7" s="19" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="B8" s="9">
-        <v>26660551242</v>
+        <v>14377439934</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="G8" s="18" t="s">
-        <v>313</v>
-      </c>
-      <c r="H8" s="2">
-        <v>16</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="K8" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>325</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="K8" s="4" t="s">
         <v>303</v>
       </c>
-      <c r="L8" s="2" t="s">
-        <v>560</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>573</v>
-      </c>
-      <c r="N8" s="2">
+      <c r="L8" s="4" t="s">
+        <v>561</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>571</v>
+      </c>
+      <c r="N8" s="4">
         <v>1</v>
       </c>
-      <c r="O8" s="21" t="s">
-        <v>366</v>
+      <c r="O8" s="11" t="s">
+        <v>373</v>
       </c>
       <c r="P8" s="21" t="s">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="Q8" s="19"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
-        <v>82</v>
+        <v>10</v>
       </c>
       <c r="B9" s="9">
-        <v>15439369480</v>
+        <v>16115748310</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>83</v>
+        <v>11</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>84</v>
+        <v>12</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>85</v>
+        <v>13</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>314</v>
+        <v>328</v>
       </c>
       <c r="H9" s="2">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>307</v>
+        <v>318</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>308</v>
+        <v>319</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>303</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>560</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>573</v>
+        <v>561</v>
+      </c>
+      <c r="M9" s="4" t="s">
+        <v>571</v>
       </c>
       <c r="N9" s="2">
         <v>1</v>
       </c>
-      <c r="O9" s="21" t="s">
-        <v>367</v>
-      </c>
-      <c r="P9" s="21" t="s">
-        <v>401</v>
-      </c>
-      <c r="Q9" s="20"/>
+      <c r="O9" s="11" t="s">
+        <v>374</v>
+      </c>
+      <c r="P9" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="Q9" s="19"/>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="12" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="B10" s="9">
-        <v>6734916496</v>
+        <v>10364360046</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>88</v>
+        <v>108</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>89</v>
+        <v>109</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="H10" s="2">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>307</v>
+        <v>318</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>308</v>
+        <v>319</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>303</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>560</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>573</v>
+        <v>561</v>
+      </c>
+      <c r="M10" s="4" t="s">
+        <v>571</v>
       </c>
       <c r="N10" s="2">
         <v>1</v>
       </c>
       <c r="O10" s="11" t="s">
-        <v>368</v>
-      </c>
-      <c r="P10" s="21" t="s">
-        <v>402</v>
-      </c>
-      <c r="Q10" s="19" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+        <v>375</v>
+      </c>
+      <c r="P10" s="11" t="s">
+        <v>409</v>
+      </c>
+      <c r="Q10" s="19"/>
+    </row>
+    <row r="11" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="12" t="s">
-        <v>5</v>
+        <v>120</v>
       </c>
       <c r="B11" s="9">
-        <v>10562161590</v>
+        <v>8858774682</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>8</v>
+        <v>122</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="G11" s="18" t="s">
-        <v>316</v>
+        <v>123</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>336</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>318</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>319</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>309</v>
-      </c>
-      <c r="L11" s="4" t="s">
-        <v>561</v>
-      </c>
-      <c r="M11" s="4" t="s">
-        <v>571</v>
-      </c>
-      <c r="N11" s="4">
-        <v>1</v>
+        <v>337</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="L11" s="5" t="s">
+        <v>566</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>572</v>
+      </c>
+      <c r="N11" s="5">
+        <v>2</v>
       </c>
       <c r="O11" s="11" t="s">
-        <v>369</v>
+        <v>379</v>
       </c>
       <c r="P11" s="21" t="s">
-        <v>403</v>
+        <v>413</v>
       </c>
       <c r="Q11" s="19"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
-        <v>90</v>
+        <v>124</v>
       </c>
       <c r="B12" s="9">
-        <v>13343108054</v>
+        <v>11407765818</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>91</v>
+        <v>125</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>92</v>
+        <v>126</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>93</v>
+        <v>127</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>320</v>
+        <v>338</v>
       </c>
       <c r="H12" s="2">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>570</v>
+        <v>566</v>
+      </c>
+      <c r="M12" s="5" t="s">
+        <v>572</v>
       </c>
       <c r="N12" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O12" s="11" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
       <c r="P12" s="11" t="s">
-        <v>404</v>
+        <v>414</v>
       </c>
       <c r="Q12" s="19"/>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" s="12" t="s">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="B13" s="9">
-        <v>10476325640</v>
+        <v>13085650940</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>96</v>
+        <v>134</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>97</v>
+        <v>135</v>
       </c>
       <c r="G13" s="18" t="s">
-        <v>323</v>
+        <v>340</v>
       </c>
       <c r="H13" s="2">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>318</v>
+        <v>331</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>319</v>
+        <v>332</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>561</v>
-      </c>
-      <c r="M13" s="4" t="s">
-        <v>571</v>
+        <v>566</v>
+      </c>
+      <c r="M13" s="5" t="s">
+        <v>572</v>
       </c>
       <c r="N13" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O13" s="11" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="P13" s="11" t="s">
-        <v>405</v>
+        <v>416</v>
       </c>
       <c r="Q13" s="19"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
-        <v>98</v>
+        <v>18</v>
       </c>
       <c r="B14" s="9">
-        <v>18451790186</v>
+        <v>20970644138</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>99</v>
+        <v>19</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>101</v>
+        <v>21</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>324</v>
+        <v>346</v>
       </c>
       <c r="H14" s="2">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>318</v>
+        <v>342</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>319</v>
+        <v>343</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>561</v>
-      </c>
-      <c r="M14" s="4" t="s">
-        <v>571</v>
+        <v>567</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>574</v>
       </c>
       <c r="N14" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O14" s="21" t="s">
-        <v>372</v>
+        <v>386</v>
       </c>
       <c r="P14" s="11" t="s">
-        <v>406</v>
+        <v>420</v>
       </c>
       <c r="Q14" s="19"/>
     </row>
-    <row r="15" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
-        <v>102</v>
+        <v>22</v>
       </c>
       <c r="B15" s="9">
-        <v>14377439934</v>
+        <v>12472888410</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>103</v>
+        <v>23</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>104</v>
+        <v>24</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>325</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>326</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>318</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>319</v>
-      </c>
-      <c r="K15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="H15" s="2">
+        <v>35</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="K15" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="L15" s="4" t="s">
-        <v>561</v>
-      </c>
-      <c r="M15" s="4" t="s">
-        <v>571</v>
-      </c>
-      <c r="N15" s="4">
-        <v>1</v>
+      <c r="L15" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="N15" s="2">
+        <v>2</v>
       </c>
       <c r="O15" s="11" t="s">
-        <v>373</v>
-      </c>
-      <c r="P15" s="21" t="s">
-        <v>407</v>
-      </c>
-      <c r="Q15" s="19"/>
+        <v>387</v>
+      </c>
+      <c r="P15" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="Q15" s="20"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16" s="12" t="s">
-        <v>10</v>
+        <v>144</v>
       </c>
       <c r="B16" s="9">
-        <v>16115748310</v>
+        <v>10482402182</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>11</v>
+        <v>145</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>12</v>
+        <v>146</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>13</v>
+        <v>147</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>328</v>
+        <v>348</v>
       </c>
       <c r="H16" s="2">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>318</v>
+        <v>342</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>319</v>
+        <v>343</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>303</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>561</v>
-      </c>
-      <c r="M16" s="4" t="s">
-        <v>571</v>
+        <v>567</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>574</v>
       </c>
       <c r="N16" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O16" s="11" t="s">
-        <v>374</v>
+        <v>388</v>
       </c>
       <c r="P16" s="11" t="s">
-        <v>408</v>
+        <v>422</v>
       </c>
       <c r="Q16" s="19"/>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17" s="12" t="s">
-        <v>106</v>
+        <v>160</v>
       </c>
       <c r="B17" s="9">
-        <v>10364360046</v>
+        <v>8597671522</v>
       </c>
       <c r="C17" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>107</v>
+        <v>161</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>108</v>
+        <v>162</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>109</v>
+        <v>163</v>
       </c>
       <c r="G17" s="18" t="s">
-        <v>327</v>
+        <v>355</v>
       </c>
       <c r="H17" s="2">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>318</v>
+        <v>350</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>319</v>
+        <v>351</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>303</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>561</v>
-      </c>
-      <c r="M17" s="4" t="s">
-        <v>571</v>
+        <v>568</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>574</v>
       </c>
       <c r="N17" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O17" s="11" t="s">
-        <v>375</v>
+        <v>393</v>
       </c>
       <c r="P17" s="11" t="s">
-        <v>409</v>
+        <v>427</v>
       </c>
       <c r="Q17" s="19"/>
     </row>
-    <row r="18" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A18" s="12" t="s">
-        <v>110</v>
+        <v>164</v>
       </c>
       <c r="B18" s="9">
-        <v>9619926120</v>
+        <v>11427089288</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>55</v>
+        <v>165</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>111</v>
+        <v>166</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>329</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>330</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="K18" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="L18" s="5" t="s">
-        <v>566</v>
-      </c>
-      <c r="M18" s="5" t="s">
-        <v>572</v>
-      </c>
-      <c r="N18" s="5">
+        <v>167</v>
+      </c>
+      <c r="G18" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="H18" s="2">
+        <v>41</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="N18" s="2">
         <v>2</v>
       </c>
       <c r="O18" s="11" t="s">
-        <v>376</v>
+        <v>394</v>
       </c>
       <c r="P18" s="11" t="s">
-        <v>410</v>
+        <v>428</v>
       </c>
       <c r="Q18" s="19"/>
     </row>
-    <row r="19" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
-        <v>112</v>
+        <v>168</v>
       </c>
       <c r="B19" s="9">
-        <v>11413688944</v>
+        <v>13353032378</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>113</v>
+        <v>169</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>114</v>
+        <v>170</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="G19" s="10" t="s">
-        <v>333</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="J19" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="K19" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="L19" s="5" t="s">
-        <v>566</v>
-      </c>
-      <c r="M19" s="5" t="s">
-        <v>572</v>
-      </c>
-      <c r="N19" s="5">
+        <v>171</v>
+      </c>
+      <c r="G19" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="H19" s="2">
+        <v>42</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="N19" s="2">
         <v>2</v>
       </c>
       <c r="O19" s="11" t="s">
-        <v>377</v>
+        <v>360</v>
       </c>
       <c r="P19" s="11" t="s">
-        <v>411</v>
+        <v>361</v>
       </c>
       <c r="Q19" s="19"/>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A20" s="12" t="s">
-        <v>116</v>
+        <v>30</v>
       </c>
       <c r="B20" s="9">
-        <v>8029463656</v>
+        <v>11056288252</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>117</v>
+        <v>31</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>118</v>
+        <v>32</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>119</v>
+        <v>33</v>
       </c>
       <c r="G20" s="18" t="s">
-        <v>335</v>
+        <v>437</v>
       </c>
       <c r="H20" s="2">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>331</v>
+        <v>433</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>332</v>
+        <v>434</v>
       </c>
       <c r="K20" s="2" t="s">
         <v>309</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>566</v>
-      </c>
-      <c r="M20" s="5" t="s">
-        <v>572</v>
+        <v>562</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>575</v>
       </c>
       <c r="N20" s="2">
         <v>2</v>
       </c>
       <c r="O20" s="11" t="s">
-        <v>378</v>
+        <v>435</v>
       </c>
       <c r="P20" s="11" t="s">
-        <v>412</v>
-      </c>
-      <c r="Q20" s="20"/>
-    </row>
-    <row r="21" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+      <c r="Q20" s="19" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A21" s="12" t="s">
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="B21" s="9">
-        <v>8858774682</v>
+        <v>9255120388</v>
       </c>
       <c r="C21" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>121</v>
+        <v>181</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>122</v>
+        <v>182</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="G21" s="10" t="s">
-        <v>336</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="I21" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="J21" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="K21" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="G21" s="18" t="s">
+        <v>443</v>
+      </c>
+      <c r="H21" s="2">
+        <v>46</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="K21" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="L21" s="5" t="s">
-        <v>566</v>
-      </c>
-      <c r="M21" s="5" t="s">
-        <v>572</v>
-      </c>
-      <c r="N21" s="5">
+      <c r="L21" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="N21" s="2">
         <v>2</v>
       </c>
       <c r="O21" s="11" t="s">
-        <v>379</v>
-      </c>
-      <c r="P21" s="21" t="s">
-        <v>413</v>
+        <v>441</v>
+      </c>
+      <c r="P21" s="11" t="s">
+        <v>442</v>
       </c>
       <c r="Q21" s="19"/>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A22" s="12" t="s">
-        <v>124</v>
+        <v>184</v>
       </c>
       <c r="B22" s="9">
-        <v>11407765818</v>
+        <v>16518497020</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>125</v>
+        <v>185</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>126</v>
+        <v>186</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>127</v>
+        <v>187</v>
       </c>
       <c r="G22" s="18" t="s">
-        <v>338</v>
+        <v>446</v>
       </c>
       <c r="H22" s="2">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>331</v>
+        <v>433</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>332</v>
+        <v>434</v>
       </c>
       <c r="K22" s="2" t="s">
         <v>303</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>566</v>
-      </c>
-      <c r="M22" s="5" t="s">
-        <v>572</v>
+        <v>562</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>575</v>
       </c>
       <c r="N22" s="2">
         <v>2</v>
       </c>
       <c r="O22" s="11" t="s">
-        <v>380</v>
+        <v>444</v>
       </c>
       <c r="P22" s="11" t="s">
-        <v>414</v>
+        <v>445</v>
       </c>
       <c r="Q22" s="19"/>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
-        <v>128</v>
+        <v>188</v>
       </c>
       <c r="B23" s="9">
-        <v>21439362030</v>
+        <v>9063966770</v>
       </c>
       <c r="C23" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>129</v>
+        <v>189</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>130</v>
+        <v>190</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>131</v>
+        <v>191</v>
       </c>
       <c r="G23" s="18" t="s">
-        <v>339</v>
+        <v>449</v>
       </c>
       <c r="H23" s="2">
+        <v>48</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="N23" s="2">
         <v>2</v>
       </c>
-      <c r="I23" s="2" t="s">
-        <v>321</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="L23" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="M23" s="2" t="s">
-        <v>570</v>
-      </c>
-      <c r="N23" s="2">
-        <v>1</v>
-      </c>
       <c r="O23" s="11" t="s">
-        <v>381</v>
+        <v>447</v>
       </c>
       <c r="P23" s="11" t="s">
-        <v>415</v>
+        <v>448</v>
       </c>
       <c r="Q23" s="19"/>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A24" s="12" t="s">
-        <v>132</v>
+        <v>34</v>
       </c>
       <c r="B24" s="9">
-        <v>13085650940</v>
+        <v>20171437076</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>133</v>
+        <v>35</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>134</v>
+        <v>36</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>135</v>
+        <v>37</v>
       </c>
       <c r="G24" s="18" t="s">
-        <v>340</v>
+        <v>456</v>
       </c>
       <c r="H24" s="2">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>332</v>
+        <v>322</v>
       </c>
       <c r="K24" s="2" t="s">
         <v>303</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>566</v>
-      </c>
-      <c r="M24" s="5" t="s">
-        <v>572</v>
+        <v>558</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>570</v>
       </c>
       <c r="N24" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O24" s="11" t="s">
-        <v>382</v>
+        <v>454</v>
       </c>
       <c r="P24" s="11" t="s">
-        <v>416</v>
+        <v>455</v>
       </c>
       <c r="Q24" s="19"/>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
-        <v>136</v>
+        <v>204</v>
       </c>
       <c r="B25" s="9">
-        <v>12524592018</v>
+        <v>10592598358</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>137</v>
+        <v>205</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>138</v>
+        <v>206</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>139</v>
+        <v>207</v>
       </c>
       <c r="G25" s="18" t="s">
-        <v>341</v>
+        <v>466</v>
       </c>
       <c r="H25" s="2">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>342</v>
+        <v>453</v>
       </c>
       <c r="J25" s="2" t="s">
         <v>343</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>567</v>
+        <v>563</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="N25" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O25" s="11" t="s">
-        <v>383</v>
+        <v>465</v>
       </c>
       <c r="P25" s="11" t="s">
-        <v>417</v>
+        <v>464</v>
       </c>
       <c r="Q25" s="19"/>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
-        <v>140</v>
+        <v>208</v>
       </c>
       <c r="B26" s="9">
-        <v>7940536736</v>
+        <v>10264253388</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>141</v>
+        <v>209</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>142</v>
+        <v>210</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>143</v>
+        <v>211</v>
       </c>
       <c r="G26" s="18" t="s">
-        <v>344</v>
+        <v>469</v>
       </c>
       <c r="H26" s="2">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>342</v>
+        <v>453</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>343</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>567</v>
+        <v>563</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="N26" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O26" s="11" t="s">
-        <v>384</v>
-      </c>
-      <c r="P26" s="21" t="s">
-        <v>418</v>
+        <v>467</v>
+      </c>
+      <c r="P26" s="11" t="s">
+        <v>468</v>
       </c>
       <c r="Q26" s="19"/>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A27" s="12" t="s">
-        <v>14</v>
+        <v>212</v>
       </c>
       <c r="B27" s="9">
-        <v>9355760378</v>
+        <v>11552323856</v>
       </c>
       <c r="C27" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>15</v>
+        <v>213</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>16</v>
+        <v>214</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>17</v>
+        <v>215</v>
       </c>
       <c r="G27" s="18" t="s">
-        <v>345</v>
+        <v>472</v>
       </c>
       <c r="H27" s="2">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>342</v>
+        <v>453</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>343</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>567</v>
+        <v>563</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="N27" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O27" s="11" t="s">
-        <v>385</v>
+        <v>470</v>
       </c>
       <c r="P27" s="11" t="s">
-        <v>419</v>
-      </c>
-      <c r="Q27" s="20"/>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+        <v>471</v>
+      </c>
+      <c r="Q27" s="19"/>
+    </row>
+    <row r="28" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="12" t="s">
-        <v>18</v>
+        <v>224</v>
       </c>
       <c r="B28" s="9">
-        <v>20970644138</v>
+        <v>18537630364</v>
       </c>
       <c r="C28" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>19</v>
+        <v>225</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>20</v>
+        <v>226</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G28" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="H28" s="2">
-        <v>34</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>343</v>
-      </c>
-      <c r="K28" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="G28" s="10" t="s">
+        <v>485</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>476</v>
+      </c>
+      <c r="J28" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="K28" s="6" t="s">
         <v>303</v>
       </c>
-      <c r="L28" s="2" t="s">
-        <v>567</v>
+      <c r="L28" s="6" t="s">
+        <v>564</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>574</v>
-      </c>
-      <c r="N28" s="2">
-        <v>2</v>
-      </c>
-      <c r="O28" s="21" t="s">
-        <v>386</v>
+        <v>577</v>
+      </c>
+      <c r="N28" s="6">
+        <v>3</v>
+      </c>
+      <c r="O28" s="11" t="s">
+        <v>483</v>
       </c>
       <c r="P28" s="11" t="s">
-        <v>420</v>
+        <v>484</v>
       </c>
       <c r="Q28" s="19"/>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A29" s="12" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="B29" s="9">
-        <v>12472888410</v>
+        <v>10763218090</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>23</v>
+        <v>229</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>24</v>
+        <v>230</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>25</v>
+        <v>231</v>
       </c>
       <c r="G29" s="18" t="s">
-        <v>347</v>
+        <v>489</v>
       </c>
       <c r="H29" s="2">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>342</v>
+        <v>476</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>343</v>
+        <v>322</v>
       </c>
       <c r="K29" s="2" t="s">
         <v>303</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="N29" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O29" s="11" t="s">
-        <v>387</v>
+        <v>487</v>
       </c>
       <c r="P29" s="11" t="s">
-        <v>421</v>
-      </c>
-      <c r="Q29" s="20"/>
+        <v>488</v>
+      </c>
+      <c r="Q29" s="19"/>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A30" s="12" t="s">
-        <v>144</v>
+        <v>232</v>
       </c>
       <c r="B30" s="9">
-        <v>10482402182</v>
+        <v>19481335366</v>
       </c>
       <c r="C30" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>145</v>
+        <v>233</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>146</v>
+        <v>234</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>147</v>
+        <v>235</v>
       </c>
       <c r="G30" s="18" t="s">
-        <v>348</v>
+        <v>492</v>
       </c>
       <c r="H30" s="2">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>342</v>
+        <v>321</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>343</v>
+        <v>322</v>
       </c>
       <c r="K30" s="2" t="s">
         <v>303</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>567</v>
+        <v>558</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>574</v>
+        <v>570</v>
       </c>
       <c r="N30" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O30" s="11" t="s">
-        <v>388</v>
+        <v>490</v>
       </c>
       <c r="P30" s="11" t="s">
-        <v>422</v>
+        <v>491</v>
       </c>
       <c r="Q30" s="19"/>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A31" s="12" t="s">
-        <v>148</v>
+        <v>236</v>
       </c>
       <c r="B31" s="9">
-        <v>13842085138</v>
+        <v>7436774160</v>
       </c>
       <c r="C31" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>149</v>
+        <v>237</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>150</v>
+        <v>238</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>151</v>
+        <v>239</v>
       </c>
       <c r="G31" s="18" t="s">
-        <v>349</v>
+        <v>495</v>
       </c>
       <c r="H31" s="2">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>350</v>
+        <v>476</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>351</v>
+        <v>322</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>568</v>
+        <v>564</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="N31" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O31" s="11" t="s">
-        <v>389</v>
+        <v>493</v>
       </c>
       <c r="P31" s="11" t="s">
-        <v>423</v>
+        <v>494</v>
       </c>
       <c r="Q31" s="19"/>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A32" s="12" t="s">
-        <v>26</v>
+        <v>252</v>
       </c>
       <c r="B32" s="9">
-        <v>8067526528</v>
+        <v>7765687192</v>
       </c>
       <c r="C32" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>27</v>
+        <v>253</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>28</v>
+        <v>254</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>29</v>
+        <v>255</v>
       </c>
       <c r="G32" s="18" t="s">
-        <v>352</v>
+        <v>510</v>
       </c>
       <c r="H32" s="2">
-        <v>38</v>
+        <v>64</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>350</v>
+        <v>499</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>351</v>
+        <v>500</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="N32" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O32" s="11" t="s">
-        <v>390</v>
+        <v>508</v>
       </c>
       <c r="P32" s="11" t="s">
-        <v>424</v>
+        <v>509</v>
       </c>
       <c r="Q32" s="19"/>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A33" s="12" t="s">
-        <v>152</v>
+        <v>256</v>
       </c>
       <c r="B33" s="9">
-        <v>10707474024</v>
+        <v>13710075502</v>
       </c>
       <c r="C33" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>153</v>
+        <v>257</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>154</v>
+        <v>258</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>155</v>
+        <v>259</v>
       </c>
       <c r="G33" s="18" t="s">
-        <v>353</v>
+        <v>513</v>
       </c>
       <c r="H33" s="2">
-        <v>39</v>
+        <v>65</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>350</v>
+        <v>499</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>351</v>
+        <v>500</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="N33" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O33" s="11" t="s">
-        <v>391</v>
+        <v>511</v>
       </c>
       <c r="P33" s="11" t="s">
-        <v>425</v>
+        <v>512</v>
       </c>
       <c r="Q33" s="19"/>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A34" s="12" t="s">
-        <v>156</v>
+        <v>260</v>
       </c>
       <c r="B34" s="9">
-        <v>10153199532</v>
+        <v>13709651192</v>
       </c>
       <c r="C34" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>157</v>
+        <v>261</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>158</v>
+        <v>262</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>159</v>
+        <v>263</v>
       </c>
       <c r="G34" s="18" t="s">
-        <v>354</v>
+        <v>516</v>
       </c>
       <c r="H34" s="2">
+        <v>66</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="M34" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="N34" s="2">
         <v>3</v>
       </c>
-      <c r="I34" s="2" t="s">
-        <v>321</v>
-      </c>
-      <c r="J34" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="L34" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="M34" s="2" t="s">
-        <v>570</v>
-      </c>
-      <c r="N34" s="2">
-        <v>1</v>
-      </c>
       <c r="O34" s="11" t="s">
-        <v>392</v>
+        <v>514</v>
       </c>
       <c r="P34" s="11" t="s">
-        <v>426</v>
-      </c>
-      <c r="Q34" s="19" t="s">
-        <v>580</v>
-      </c>
+        <v>515</v>
+      </c>
+      <c r="Q34" s="19"/>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A35" s="12" t="s">
-        <v>160</v>
+        <v>276</v>
       </c>
       <c r="B35" s="9">
-        <v>8597671522</v>
+        <v>11103894928</v>
       </c>
       <c r="C35" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>161</v>
+        <v>277</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>162</v>
+        <v>278</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>163</v>
+        <v>279</v>
       </c>
       <c r="G35" s="18" t="s">
-        <v>355</v>
+        <v>531</v>
       </c>
       <c r="H35" s="2">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>350</v>
+        <v>321</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>351</v>
+        <v>322</v>
       </c>
       <c r="K35" s="2" t="s">
         <v>303</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>568</v>
+        <v>558</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>574</v>
+        <v>570</v>
       </c>
       <c r="N35" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O35" s="11" t="s">
-        <v>393</v>
+        <v>529</v>
       </c>
       <c r="P35" s="11" t="s">
-        <v>427</v>
+        <v>530</v>
       </c>
       <c r="Q35" s="19"/>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A36" s="12" t="s">
-        <v>164</v>
+        <v>42</v>
       </c>
       <c r="B36" s="9">
-        <v>11427089288</v>
+        <v>23573858468</v>
       </c>
       <c r="C36" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>165</v>
+        <v>43</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>166</v>
+        <v>44</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>167</v>
+        <v>45</v>
       </c>
       <c r="G36" s="18" t="s">
-        <v>359</v>
+        <v>534</v>
       </c>
       <c r="H36" s="2">
-        <v>41</v>
+        <v>70</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>350</v>
+        <v>521</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>351</v>
+        <v>522</v>
       </c>
       <c r="K36" s="2" t="s">
         <v>303</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>568</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>574</v>
+        <v>565</v>
+      </c>
+      <c r="M36" s="4" t="s">
+        <v>579</v>
       </c>
       <c r="N36" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O36" s="11" t="s">
-        <v>394</v>
+        <v>532</v>
       </c>
       <c r="P36" s="11" t="s">
-        <v>428</v>
-      </c>
-      <c r="Q36" s="19"/>
+        <v>533</v>
+      </c>
+      <c r="Q36" s="19" t="s">
+        <v>552</v>
+      </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A37" s="12" t="s">
-        <v>168</v>
+        <v>46</v>
       </c>
       <c r="B37" s="9">
-        <v>13353032378</v>
+        <v>27406244206</v>
       </c>
       <c r="C37" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>169</v>
+        <v>47</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>170</v>
+        <v>48</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>171</v>
+        <v>49</v>
       </c>
       <c r="G37" s="18" t="s">
-        <v>429</v>
+        <v>537</v>
       </c>
       <c r="H37" s="2">
-        <v>42</v>
+        <v>71</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>350</v>
+        <v>521</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>351</v>
+        <v>522</v>
       </c>
       <c r="K37" s="2" t="s">
         <v>303</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>568</v>
-      </c>
-      <c r="M37" s="2" t="s">
-        <v>574</v>
+        <v>565</v>
+      </c>
+      <c r="M37" s="4" t="s">
+        <v>579</v>
       </c>
       <c r="N37" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O37" s="11" t="s">
-        <v>360</v>
+        <v>535</v>
       </c>
       <c r="P37" s="11" t="s">
-        <v>361</v>
-      </c>
-      <c r="Q37" s="19"/>
+        <v>536</v>
+      </c>
+      <c r="Q37" s="19" t="s">
+        <v>553</v>
+      </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A38" s="12" t="s">
-        <v>172</v>
+        <v>280</v>
       </c>
       <c r="B38" s="9">
-        <v>9423474214</v>
+        <v>13458064958</v>
       </c>
       <c r="C38" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>173</v>
+        <v>281</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>174</v>
+        <v>282</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>175</v>
+        <v>283</v>
       </c>
       <c r="G38" s="18" t="s">
-        <v>432</v>
+        <v>551</v>
       </c>
       <c r="H38" s="2">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>433</v>
+        <v>521</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>434</v>
+        <v>522</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>562</v>
-      </c>
-      <c r="M38" s="2" t="s">
-        <v>575</v>
+        <v>565</v>
+      </c>
+      <c r="M38" s="4" t="s">
+        <v>579</v>
       </c>
       <c r="N38" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O38" s="11" t="s">
-        <v>430</v>
+        <v>538</v>
       </c>
       <c r="P38" s="11" t="s">
-        <v>431</v>
-      </c>
-      <c r="Q38" s="19"/>
+        <v>539</v>
+      </c>
+      <c r="Q38" s="19" t="s">
+        <v>554</v>
+      </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A39" s="12" t="s">
-        <v>30</v>
+        <v>66</v>
       </c>
       <c r="B39" s="9">
-        <v>11056288252</v>
+        <v>9412089720</v>
       </c>
       <c r="C39" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="G39" s="18" t="s">
-        <v>437</v>
+        <v>306</v>
       </c>
       <c r="H39" s="2">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>433</v>
+        <v>307</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>434</v>
+        <v>308</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="N39" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O39" s="11" t="s">
-        <v>435</v>
+        <v>363</v>
       </c>
       <c r="P39" s="11" t="s">
-        <v>436</v>
-      </c>
-      <c r="Q39" s="19" t="s">
-        <v>583</v>
-      </c>
-    </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
+        <v>397</v>
+      </c>
+      <c r="Q39" s="19"/>
+    </row>
+    <row r="40" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A40" s="12" t="s">
-        <v>176</v>
+        <v>70</v>
       </c>
       <c r="B40" s="9">
-        <v>8401074958</v>
+        <v>9959631122</v>
       </c>
       <c r="C40" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>177</v>
+        <v>71</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>178</v>
+        <v>72</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="G40" s="18" t="s">
-        <v>440</v>
-      </c>
-      <c r="H40" s="2">
-        <v>45</v>
-      </c>
-      <c r="I40" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="J40" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="K40" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G40" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="K40" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="L40" s="2" t="s">
-        <v>562</v>
-      </c>
-      <c r="M40" s="2" t="s">
-        <v>575</v>
-      </c>
-      <c r="N40" s="2">
-        <v>2</v>
+      <c r="L40" s="3" t="s">
+        <v>560</v>
+      </c>
+      <c r="M40" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="N40" s="3">
+        <v>1</v>
       </c>
       <c r="O40" s="11" t="s">
-        <v>438</v>
+        <v>364</v>
       </c>
       <c r="P40" s="11" t="s">
-        <v>439</v>
+        <v>398</v>
       </c>
       <c r="Q40" s="19"/>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A41" s="12" t="s">
-        <v>180</v>
+        <v>74</v>
       </c>
       <c r="B41" s="9">
-        <v>9255120388</v>
+        <v>12797457172</v>
       </c>
       <c r="C41" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>181</v>
+        <v>75</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>182</v>
+        <v>76</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>183</v>
+        <v>77</v>
       </c>
       <c r="G41" s="18" t="s">
-        <v>443</v>
+        <v>312</v>
       </c>
       <c r="H41" s="2">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>433</v>
+        <v>307</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>434</v>
+        <v>308</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>562</v>
-      </c>
-      <c r="M41" s="2" t="s">
-        <v>575</v>
+        <v>560</v>
+      </c>
+      <c r="M41" s="1" t="s">
+        <v>573</v>
       </c>
       <c r="N41" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O41" s="11" t="s">
-        <v>441</v>
+        <v>365</v>
       </c>
       <c r="P41" s="11" t="s">
-        <v>442</v>
+        <v>399</v>
       </c>
       <c r="Q41" s="19"/>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A42" s="12" t="s">
-        <v>184</v>
+        <v>5</v>
       </c>
       <c r="B42" s="9">
-        <v>16518497020</v>
+        <v>10562161590</v>
       </c>
       <c r="C42" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>185</v>
+        <v>7</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>186</v>
+        <v>8</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>187</v>
+        <v>9</v>
       </c>
       <c r="G42" s="18" t="s">
-        <v>446</v>
-      </c>
-      <c r="H42" s="2">
-        <v>47</v>
-      </c>
-      <c r="I42" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="J42" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="K42" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="L42" s="2" t="s">
-        <v>562</v>
-      </c>
-      <c r="M42" s="2" t="s">
-        <v>575</v>
-      </c>
-      <c r="N42" s="2">
-        <v>2</v>
+        <v>316</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="I42" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="J42" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="K42" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="L42" s="4" t="s">
+        <v>561</v>
+      </c>
+      <c r="M42" s="4" t="s">
+        <v>571</v>
+      </c>
+      <c r="N42" s="4">
+        <v>1</v>
       </c>
       <c r="O42" s="11" t="s">
-        <v>444</v>
-      </c>
-      <c r="P42" s="11" t="s">
-        <v>445</v>
+        <v>369</v>
+      </c>
+      <c r="P42" s="21" t="s">
+        <v>403</v>
       </c>
       <c r="Q42" s="19"/>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A43" s="12" t="s">
-        <v>188</v>
+        <v>90</v>
       </c>
       <c r="B43" s="9">
-        <v>9063966770</v>
+        <v>13343108054</v>
       </c>
       <c r="C43" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>189</v>
+        <v>91</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>190</v>
+        <v>92</v>
       </c>
       <c r="F43" s="9" t="s">
-        <v>191</v>
+        <v>93</v>
       </c>
       <c r="G43" s="18" t="s">
-        <v>449</v>
+        <v>320</v>
       </c>
       <c r="H43" s="2">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>433</v>
+        <v>321</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>434</v>
+        <v>322</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>562</v>
+        <v>558</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>575</v>
+        <v>570</v>
       </c>
       <c r="N43" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O43" s="11" t="s">
-        <v>447</v>
+        <v>370</v>
       </c>
       <c r="P43" s="11" t="s">
-        <v>448</v>
+        <v>404</v>
       </c>
       <c r="Q43" s="19"/>
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A44" s="12" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
       <c r="B44" s="9">
-        <v>14389645264</v>
+        <v>10476325640</v>
       </c>
       <c r="C44" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>193</v>
+        <v>95</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>194</v>
+        <v>96</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>195</v>
+        <v>97</v>
       </c>
       <c r="G44" s="18" t="s">
-        <v>452</v>
+        <v>323</v>
       </c>
       <c r="H44" s="2">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>453</v>
+        <v>318</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>343</v>
+        <v>319</v>
       </c>
       <c r="K44" s="2" t="s">
         <v>309</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>563</v>
-      </c>
-      <c r="M44" s="2" t="s">
-        <v>576</v>
+        <v>561</v>
+      </c>
+      <c r="M44" s="4" t="s">
+        <v>571</v>
       </c>
       <c r="N44" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O44" s="11" t="s">
-        <v>450</v>
+        <v>371</v>
       </c>
       <c r="P44" s="11" t="s">
-        <v>451</v>
+        <v>405</v>
       </c>
       <c r="Q44" s="19"/>
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A45" s="12" t="s">
-        <v>34</v>
+        <v>98</v>
       </c>
       <c r="B45" s="9">
-        <v>20171437076</v>
+        <v>18451790186</v>
       </c>
       <c r="C45" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>35</v>
+        <v>99</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>36</v>
+        <v>100</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>37</v>
+        <v>101</v>
       </c>
       <c r="G45" s="18" t="s">
-        <v>456</v>
+        <v>324</v>
       </c>
       <c r="H45" s="2">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="M45" s="2" t="s">
-        <v>570</v>
+        <v>561</v>
+      </c>
+      <c r="M45" s="4" t="s">
+        <v>571</v>
       </c>
       <c r="N45" s="2">
         <v>1</v>
       </c>
-      <c r="O45" s="11" t="s">
-        <v>454</v>
+      <c r="O45" s="21" t="s">
+        <v>372</v>
       </c>
       <c r="P45" s="11" t="s">
-        <v>455</v>
+        <v>406</v>
       </c>
       <c r="Q45" s="19"/>
     </row>
     <row r="46" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A46" s="12" t="s">
-        <v>196</v>
+        <v>110</v>
       </c>
       <c r="B46" s="9">
-        <v>9849392062</v>
+        <v>9619926120</v>
       </c>
       <c r="C46" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>197</v>
+        <v>55</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>198</v>
+        <v>111</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>199</v>
+        <v>57</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>459</v>
+        <v>329</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>460</v>
+        <v>330</v>
       </c>
       <c r="I46" s="5" t="s">
-        <v>453</v>
+        <v>331</v>
       </c>
       <c r="J46" s="5" t="s">
-        <v>343</v>
+        <v>332</v>
       </c>
       <c r="K46" s="5" t="s">
         <v>309</v>
       </c>
       <c r="L46" s="5" t="s">
-        <v>563</v>
-      </c>
-      <c r="M46" s="2" t="s">
-        <v>576</v>
+        <v>566</v>
+      </c>
+      <c r="M46" s="5" t="s">
+        <v>572</v>
       </c>
       <c r="N46" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O46" s="11" t="s">
-        <v>457</v>
+        <v>376</v>
       </c>
       <c r="P46" s="11" t="s">
-        <v>458</v>
+        <v>410</v>
       </c>
       <c r="Q46" s="19"/>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A47" s="12" t="s">
-        <v>200</v>
+        <v>112</v>
       </c>
       <c r="B47" s="9">
-        <v>11144366552</v>
+        <v>11413688944</v>
       </c>
       <c r="C47" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>201</v>
+        <v>113</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>202</v>
+        <v>114</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="G47" s="18" t="s">
-        <v>463</v>
-      </c>
-      <c r="H47" s="2">
-        <v>51</v>
-      </c>
-      <c r="I47" s="2" t="s">
-        <v>453</v>
-      </c>
-      <c r="J47" s="2" t="s">
-        <v>343</v>
-      </c>
-      <c r="K47" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="G47" s="10" t="s">
+        <v>333</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="I47" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="J47" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="K47" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="L47" s="2" t="s">
-        <v>563</v>
-      </c>
-      <c r="M47" s="2" t="s">
-        <v>576</v>
-      </c>
-      <c r="N47" s="2">
-        <v>3</v>
+      <c r="L47" s="5" t="s">
+        <v>566</v>
+      </c>
+      <c r="M47" s="5" t="s">
+        <v>572</v>
+      </c>
+      <c r="N47" s="5">
+        <v>2</v>
       </c>
       <c r="O47" s="11" t="s">
-        <v>461</v>
+        <v>377</v>
       </c>
       <c r="P47" s="11" t="s">
-        <v>462</v>
+        <v>411</v>
       </c>
       <c r="Q47" s="19"/>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A48" s="12" t="s">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="B48" s="9">
-        <v>10592598358</v>
+        <v>8029463656</v>
       </c>
       <c r="C48" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>205</v>
+        <v>117</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>206</v>
+        <v>118</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>207</v>
+        <v>119</v>
       </c>
       <c r="G48" s="18" t="s">
-        <v>466</v>
+        <v>335</v>
       </c>
       <c r="H48" s="2">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>453</v>
+        <v>331</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>343</v>
+        <v>332</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>563</v>
-      </c>
-      <c r="M48" s="2" t="s">
-        <v>576</v>
+        <v>566</v>
+      </c>
+      <c r="M48" s="5" t="s">
+        <v>572</v>
       </c>
       <c r="N48" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O48" s="11" t="s">
-        <v>465</v>
+        <v>378</v>
       </c>
       <c r="P48" s="11" t="s">
-        <v>464</v>
-      </c>
-      <c r="Q48" s="19"/>
+        <v>412</v>
+      </c>
+      <c r="Q48" s="20"/>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A49" s="12" t="s">
-        <v>208</v>
+        <v>128</v>
       </c>
       <c r="B49" s="9">
-        <v>10264253388</v>
+        <v>21439362030</v>
       </c>
       <c r="C49" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>209</v>
+        <v>129</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>210</v>
+        <v>130</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>211</v>
+        <v>131</v>
       </c>
       <c r="G49" s="18" t="s">
-        <v>469</v>
+        <v>339</v>
       </c>
       <c r="H49" s="2">
-        <v>53</v>
+        <v>2</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>453</v>
+        <v>321</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>343</v>
+        <v>322</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L49" s="2" t="s">
-        <v>563</v>
+        <v>558</v>
       </c>
       <c r="M49" s="2" t="s">
-        <v>576</v>
+        <v>570</v>
       </c>
       <c r="N49" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O49" s="11" t="s">
-        <v>467</v>
+        <v>381</v>
       </c>
       <c r="P49" s="11" t="s">
-        <v>468</v>
+        <v>415</v>
       </c>
       <c r="Q49" s="19"/>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A50" s="12" t="s">
-        <v>212</v>
+        <v>136</v>
       </c>
       <c r="B50" s="9">
-        <v>11552323856</v>
+        <v>12524592018</v>
       </c>
       <c r="C50" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>213</v>
+        <v>137</v>
       </c>
       <c r="E50" s="9" t="s">
-        <v>214</v>
+        <v>138</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>215</v>
+        <v>139</v>
       </c>
       <c r="G50" s="18" t="s">
-        <v>472</v>
+        <v>341</v>
       </c>
       <c r="H50" s="2">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>453</v>
+        <v>342</v>
       </c>
       <c r="J50" s="2" t="s">
         <v>343</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="N50" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O50" s="11" t="s">
-        <v>470</v>
+        <v>383</v>
       </c>
       <c r="P50" s="11" t="s">
-        <v>471</v>
+        <v>417</v>
       </c>
       <c r="Q50" s="19"/>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A51" s="12" t="s">
-        <v>38</v>
+        <v>140</v>
       </c>
       <c r="B51" s="9">
-        <v>10592750868</v>
+        <v>7940536736</v>
       </c>
       <c r="C51" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>39</v>
+        <v>141</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>40</v>
+        <v>142</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>41</v>
+        <v>143</v>
       </c>
       <c r="G51" s="18" t="s">
-        <v>475</v>
+        <v>344</v>
       </c>
       <c r="H51" s="2">
-        <v>55</v>
+        <v>32</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>476</v>
+        <v>342</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>322</v>
+        <v>343</v>
       </c>
       <c r="K51" s="2" t="s">
         <v>309</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="N51" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O51" s="11" t="s">
-        <v>473</v>
-      </c>
-      <c r="P51" s="11" t="s">
-        <v>474</v>
+        <v>384</v>
+      </c>
+      <c r="P51" s="21" t="s">
+        <v>418</v>
       </c>
       <c r="Q51" s="19"/>
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A52" s="12" t="s">
-        <v>216</v>
+        <v>14</v>
       </c>
       <c r="B52" s="9">
-        <v>11426695178</v>
+        <v>9355760378</v>
       </c>
       <c r="C52" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>217</v>
+        <v>15</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>218</v>
+        <v>16</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>219</v>
+        <v>17</v>
       </c>
       <c r="G52" s="18" t="s">
-        <v>479</v>
+        <v>345</v>
       </c>
       <c r="H52" s="2">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>476</v>
+        <v>342</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>322</v>
+        <v>343</v>
       </c>
       <c r="K52" s="2" t="s">
         <v>309</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="N52" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O52" s="11" t="s">
-        <v>477</v>
+        <v>385</v>
       </c>
       <c r="P52" s="11" t="s">
-        <v>478</v>
-      </c>
-      <c r="Q52" s="19"/>
+        <v>419</v>
+      </c>
+      <c r="Q52" s="20"/>
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A53" s="12" t="s">
-        <v>220</v>
+        <v>148</v>
       </c>
       <c r="B53" s="9">
-        <v>7977101386</v>
+        <v>13842085138</v>
       </c>
       <c r="C53" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>221</v>
+        <v>149</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>222</v>
+        <v>150</v>
       </c>
       <c r="F53" s="9" t="s">
-        <v>223</v>
+        <v>151</v>
       </c>
       <c r="G53" s="18" t="s">
-        <v>482</v>
+        <v>349</v>
       </c>
       <c r="H53" s="2">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>476</v>
+        <v>350</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>322</v>
+        <v>351</v>
       </c>
       <c r="K53" s="2" t="s">
         <v>309</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="M53" s="2" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="N53" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O53" s="11" t="s">
-        <v>480</v>
+        <v>389</v>
       </c>
       <c r="P53" s="11" t="s">
-        <v>481</v>
-      </c>
-      <c r="Q53" s="19" t="s">
-        <v>581</v>
-      </c>
-    </row>
-    <row r="54" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+        <v>423</v>
+      </c>
+      <c r="Q53" s="19"/>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A54" s="12" t="s">
-        <v>224</v>
+        <v>26</v>
       </c>
       <c r="B54" s="9">
-        <v>18537630364</v>
+        <v>8067526528</v>
       </c>
       <c r="C54" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>225</v>
+        <v>27</v>
       </c>
       <c r="E54" s="9" t="s">
-        <v>226</v>
+        <v>28</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="G54" s="10" t="s">
-        <v>485</v>
-      </c>
-      <c r="H54" s="2" t="s">
-        <v>486</v>
-      </c>
-      <c r="I54" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="J54" s="6" t="s">
-        <v>322</v>
-      </c>
-      <c r="K54" s="6" t="s">
-        <v>303</v>
-      </c>
-      <c r="L54" s="6" t="s">
-        <v>564</v>
+        <v>29</v>
+      </c>
+      <c r="G54" s="18" t="s">
+        <v>352</v>
+      </c>
+      <c r="H54" s="2">
+        <v>38</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="L54" s="2" t="s">
+        <v>568</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>577</v>
-      </c>
-      <c r="N54" s="6">
-        <v>3</v>
+        <v>574</v>
+      </c>
+      <c r="N54" s="2">
+        <v>2</v>
       </c>
       <c r="O54" s="11" t="s">
-        <v>483</v>
+        <v>390</v>
       </c>
       <c r="P54" s="11" t="s">
-        <v>484</v>
+        <v>424</v>
       </c>
       <c r="Q54" s="19"/>
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A55" s="12" t="s">
-        <v>228</v>
+        <v>152</v>
       </c>
       <c r="B55" s="9">
-        <v>10763218090</v>
+        <v>10707474024</v>
       </c>
       <c r="C55" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>229</v>
+        <v>153</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>230</v>
+        <v>154</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>231</v>
+        <v>155</v>
       </c>
       <c r="G55" s="18" t="s">
-        <v>489</v>
+        <v>353</v>
       </c>
       <c r="H55" s="2">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>476</v>
+        <v>350</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>322</v>
+        <v>351</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="N55" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O55" s="11" t="s">
-        <v>487</v>
+        <v>391</v>
       </c>
       <c r="P55" s="11" t="s">
-        <v>488</v>
+        <v>425</v>
       </c>
       <c r="Q55" s="19"/>
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A56" s="12" t="s">
-        <v>232</v>
+        <v>156</v>
       </c>
       <c r="B56" s="9">
-        <v>19481335366</v>
+        <v>10153199532</v>
       </c>
       <c r="C56" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>233</v>
+        <v>157</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>234</v>
+        <v>158</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>235</v>
+        <v>159</v>
       </c>
       <c r="G56" s="18" t="s">
-        <v>492</v>
+        <v>354</v>
       </c>
       <c r="H56" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I56" s="2" t="s">
         <v>321</v>
@@ -5778,7 +5776,7 @@
         <v>322</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L56" s="2" t="s">
         <v>558</v>
@@ -5790,306 +5788,306 @@
         <v>1</v>
       </c>
       <c r="O56" s="11" t="s">
-        <v>490</v>
+        <v>392</v>
       </c>
       <c r="P56" s="11" t="s">
-        <v>491</v>
-      </c>
-      <c r="Q56" s="19"/>
+        <v>426</v>
+      </c>
+      <c r="Q56" s="19" t="s">
+        <v>580</v>
+      </c>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A57" s="12" t="s">
-        <v>236</v>
+        <v>172</v>
       </c>
       <c r="B57" s="9">
-        <v>7436774160</v>
+        <v>9423474214</v>
       </c>
       <c r="C57" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>237</v>
+        <v>173</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>238</v>
+        <v>174</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>239</v>
+        <v>175</v>
       </c>
       <c r="G57" s="18" t="s">
-        <v>495</v>
+        <v>432</v>
       </c>
       <c r="H57" s="2">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>476</v>
+        <v>433</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>322</v>
+        <v>434</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="M57" s="2" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="N57" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O57" s="11" t="s">
-        <v>493</v>
+        <v>430</v>
       </c>
       <c r="P57" s="11" t="s">
-        <v>494</v>
+        <v>431</v>
       </c>
       <c r="Q57" s="19"/>
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A58" s="12" t="s">
-        <v>240</v>
+        <v>176</v>
       </c>
       <c r="B58" s="9">
-        <v>20739486090</v>
+        <v>8401074958</v>
       </c>
       <c r="C58" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>241</v>
+        <v>177</v>
       </c>
       <c r="E58" s="9" t="s">
-        <v>242</v>
+        <v>178</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>243</v>
+        <v>179</v>
       </c>
       <c r="G58" s="18" t="s">
-        <v>498</v>
+        <v>440</v>
       </c>
       <c r="H58" s="2">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>499</v>
+        <v>433</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>500</v>
+        <v>434</v>
       </c>
       <c r="K58" s="2" t="s">
         <v>309</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>569</v>
+        <v>562</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="N58" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O58" s="11" t="s">
-        <v>496</v>
+        <v>438</v>
       </c>
       <c r="P58" s="11" t="s">
-        <v>497</v>
+        <v>439</v>
       </c>
       <c r="Q58" s="19"/>
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A59" s="12" t="s">
-        <v>244</v>
+        <v>192</v>
       </c>
       <c r="B59" s="9">
-        <v>9489899416</v>
+        <v>14389645264</v>
       </c>
       <c r="C59" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>245</v>
+        <v>193</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>246</v>
+        <v>194</v>
       </c>
       <c r="F59" s="9" t="s">
-        <v>247</v>
+        <v>195</v>
       </c>
       <c r="G59" s="18" t="s">
-        <v>503</v>
+        <v>452</v>
       </c>
       <c r="H59" s="2">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>499</v>
+        <v>453</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>500</v>
+        <v>343</v>
       </c>
       <c r="K59" s="2" t="s">
         <v>309</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>569</v>
+        <v>563</v>
       </c>
       <c r="M59" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="N59" s="2">
         <v>3</v>
       </c>
       <c r="O59" s="11" t="s">
-        <v>501</v>
+        <v>450</v>
       </c>
       <c r="P59" s="11" t="s">
-        <v>502</v>
-      </c>
-      <c r="Q59" s="19" t="s">
-        <v>581</v>
-      </c>
-    </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.3">
+        <v>451</v>
+      </c>
+      <c r="Q59" s="19"/>
+    </row>
+    <row r="60" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A60" s="12" t="s">
-        <v>248</v>
+        <v>196</v>
       </c>
       <c r="B60" s="9">
-        <v>12485985546</v>
+        <v>9849392062</v>
       </c>
       <c r="C60" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>249</v>
+        <v>197</v>
       </c>
       <c r="E60" s="9" t="s">
-        <v>250</v>
+        <v>198</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>251</v>
-      </c>
-      <c r="G60" s="18" t="s">
-        <v>506</v>
-      </c>
-      <c r="H60" s="2">
-        <v>63</v>
-      </c>
-      <c r="I60" s="2" t="s">
-        <v>499</v>
-      </c>
-      <c r="J60" s="2" t="s">
-        <v>500</v>
-      </c>
-      <c r="K60" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G60" s="10" t="s">
+        <v>459</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="I60" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="J60" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="K60" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="L60" s="2" t="s">
-        <v>569</v>
+      <c r="L60" s="5" t="s">
+        <v>563</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>577</v>
-      </c>
-      <c r="N60" s="2">
+        <v>576</v>
+      </c>
+      <c r="N60" s="5">
         <v>3</v>
       </c>
       <c r="O60" s="11" t="s">
-        <v>504</v>
+        <v>457</v>
       </c>
       <c r="P60" s="11" t="s">
-        <v>505</v>
+        <v>458</v>
       </c>
       <c r="Q60" s="19"/>
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A61" s="12" t="s">
-        <v>252</v>
+        <v>200</v>
       </c>
       <c r="B61" s="9">
-        <v>7765687192</v>
+        <v>11144366552</v>
       </c>
       <c r="C61" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>253</v>
+        <v>201</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>254</v>
+        <v>202</v>
       </c>
       <c r="F61" s="9" t="s">
-        <v>255</v>
+        <v>203</v>
       </c>
       <c r="G61" s="18" t="s">
-        <v>510</v>
+        <v>463</v>
       </c>
       <c r="H61" s="2">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>499</v>
+        <v>453</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>500</v>
+        <v>343</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L61" s="2" t="s">
-        <v>569</v>
+        <v>563</v>
       </c>
       <c r="M61" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="N61" s="2">
         <v>3</v>
       </c>
       <c r="O61" s="11" t="s">
-        <v>508</v>
+        <v>461</v>
       </c>
       <c r="P61" s="11" t="s">
-        <v>509</v>
+        <v>462</v>
       </c>
       <c r="Q61" s="19"/>
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A62" s="12" t="s">
-        <v>256</v>
+        <v>38</v>
       </c>
       <c r="B62" s="9">
-        <v>13710075502</v>
+        <v>10592750868</v>
       </c>
       <c r="C62" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>257</v>
+        <v>39</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>258</v>
+        <v>40</v>
       </c>
       <c r="F62" s="9" t="s">
-        <v>259</v>
+        <v>41</v>
       </c>
       <c r="G62" s="18" t="s">
-        <v>513</v>
+        <v>475</v>
       </c>
       <c r="H62" s="2">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>499</v>
+        <v>476</v>
       </c>
       <c r="J62" s="2" t="s">
-        <v>500</v>
+        <v>322</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>569</v>
+        <v>564</v>
       </c>
       <c r="M62" s="2" t="s">
         <v>577</v>
@@ -6098,49 +6096,49 @@
         <v>3</v>
       </c>
       <c r="O62" s="11" t="s">
-        <v>511</v>
+        <v>473</v>
       </c>
       <c r="P62" s="11" t="s">
-        <v>512</v>
+        <v>474</v>
       </c>
       <c r="Q62" s="19"/>
     </row>
     <row r="63" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A63" s="12" t="s">
-        <v>260</v>
+        <v>216</v>
       </c>
       <c r="B63" s="9">
-        <v>13709651192</v>
+        <v>11426695178</v>
       </c>
       <c r="C63" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>261</v>
+        <v>217</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>262</v>
+        <v>218</v>
       </c>
       <c r="F63" s="9" t="s">
-        <v>263</v>
+        <v>219</v>
       </c>
       <c r="G63" s="18" t="s">
-        <v>516</v>
+        <v>479</v>
       </c>
       <c r="H63" s="2">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>499</v>
+        <v>476</v>
       </c>
       <c r="J63" s="2" t="s">
-        <v>500</v>
+        <v>322</v>
       </c>
       <c r="K63" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L63" s="2" t="s">
-        <v>569</v>
+        <v>564</v>
       </c>
       <c r="M63" s="2" t="s">
         <v>577</v>
@@ -6149,296 +6147,296 @@
         <v>3</v>
       </c>
       <c r="O63" s="11" t="s">
-        <v>514</v>
+        <v>477</v>
       </c>
       <c r="P63" s="11" t="s">
-        <v>515</v>
+        <v>478</v>
       </c>
       <c r="Q63" s="19"/>
     </row>
-    <row r="64" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A64" s="12" t="s">
-        <v>264</v>
+        <v>220</v>
       </c>
       <c r="B64" s="9">
-        <v>13539917226</v>
+        <v>7977101386</v>
       </c>
       <c r="C64" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>265</v>
+        <v>221</v>
       </c>
       <c r="E64" s="9" t="s">
-        <v>266</v>
+        <v>222</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>267</v>
-      </c>
-      <c r="G64" s="10" t="s">
-        <v>519</v>
-      </c>
-      <c r="H64" s="2" t="s">
-        <v>520</v>
-      </c>
-      <c r="I64" s="4" t="s">
-        <v>521</v>
-      </c>
-      <c r="J64" s="4" t="s">
-        <v>522</v>
-      </c>
-      <c r="K64" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="G64" s="18" t="s">
+        <v>482</v>
+      </c>
+      <c r="H64" s="2">
+        <v>57</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="J64" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="K64" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="L64" s="4" t="s">
-        <v>565</v>
-      </c>
-      <c r="M64" s="4" t="s">
-        <v>579</v>
-      </c>
-      <c r="N64" s="4">
+      <c r="L64" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="M64" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="N64" s="2">
         <v>3</v>
       </c>
       <c r="O64" s="11" t="s">
-        <v>517</v>
+        <v>480</v>
       </c>
       <c r="P64" s="11" t="s">
-        <v>518</v>
-      </c>
-      <c r="Q64" s="19"/>
+        <v>481</v>
+      </c>
+      <c r="Q64" s="19" t="s">
+        <v>581</v>
+      </c>
     </row>
     <row r="65" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A65" s="12" t="s">
-        <v>268</v>
+        <v>240</v>
       </c>
       <c r="B65" s="9">
-        <v>18323004400</v>
+        <v>20739486090</v>
       </c>
       <c r="C65" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>269</v>
+        <v>241</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>270</v>
+        <v>242</v>
       </c>
       <c r="F65" s="9" t="s">
-        <v>271</v>
+        <v>243</v>
       </c>
       <c r="G65" s="18" t="s">
-        <v>524</v>
+        <v>498</v>
       </c>
       <c r="H65" s="2">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="I65" s="2" t="s">
-        <v>521</v>
+        <v>499</v>
       </c>
       <c r="J65" s="2" t="s">
-        <v>522</v>
+        <v>500</v>
       </c>
       <c r="K65" s="2" t="s">
         <v>309</v>
       </c>
       <c r="L65" s="2" t="s">
-        <v>565</v>
-      </c>
-      <c r="M65" s="4" t="s">
-        <v>579</v>
+        <v>569</v>
+      </c>
+      <c r="M65" s="2" t="s">
+        <v>577</v>
       </c>
       <c r="N65" s="2">
         <v>3</v>
       </c>
       <c r="O65" s="11" t="s">
-        <v>507</v>
+        <v>496</v>
       </c>
       <c r="P65" s="11" t="s">
-        <v>523</v>
+        <v>497</v>
       </c>
       <c r="Q65" s="19"/>
     </row>
-    <row r="66" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A66" s="12" t="s">
-        <v>272</v>
+        <v>244</v>
       </c>
       <c r="B66" s="9">
-        <v>16388897646</v>
+        <v>9489899416</v>
       </c>
       <c r="C66" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>273</v>
+        <v>245</v>
       </c>
       <c r="E66" s="9" t="s">
-        <v>274</v>
+        <v>246</v>
       </c>
       <c r="F66" s="9" t="s">
-        <v>275</v>
-      </c>
-      <c r="G66" s="10" t="s">
-        <v>527</v>
-      </c>
-      <c r="H66" s="2" t="s">
-        <v>528</v>
-      </c>
-      <c r="I66" s="4" t="s">
-        <v>521</v>
-      </c>
-      <c r="J66" s="4" t="s">
-        <v>522</v>
-      </c>
-      <c r="K66" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="G66" s="18" t="s">
+        <v>503</v>
+      </c>
+      <c r="H66" s="2">
+        <v>62</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="J66" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="K66" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="L66" s="4" t="s">
-        <v>565</v>
-      </c>
-      <c r="M66" s="4" t="s">
-        <v>579</v>
-      </c>
-      <c r="N66" s="4">
+      <c r="L66" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="M66" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="N66" s="2">
         <v>3</v>
       </c>
       <c r="O66" s="11" t="s">
-        <v>525</v>
+        <v>501</v>
       </c>
       <c r="P66" s="11" t="s">
-        <v>526</v>
+        <v>502</v>
       </c>
       <c r="Q66" s="19" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
     </row>
     <row r="67" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A67" s="12" t="s">
-        <v>276</v>
+        <v>248</v>
       </c>
       <c r="B67" s="9">
-        <v>11103894928</v>
+        <v>12485985546</v>
       </c>
       <c r="C67" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>277</v>
+        <v>249</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>278</v>
+        <v>250</v>
       </c>
       <c r="F67" s="9" t="s">
-        <v>279</v>
+        <v>251</v>
       </c>
       <c r="G67" s="18" t="s">
-        <v>531</v>
+        <v>506</v>
       </c>
       <c r="H67" s="2">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="I67" s="2" t="s">
-        <v>321</v>
+        <v>499</v>
       </c>
       <c r="J67" s="2" t="s">
-        <v>322</v>
+        <v>500</v>
       </c>
       <c r="K67" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L67" s="2" t="s">
-        <v>558</v>
+        <v>569</v>
       </c>
       <c r="M67" s="2" t="s">
-        <v>570</v>
+        <v>577</v>
       </c>
       <c r="N67" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O67" s="11" t="s">
-        <v>529</v>
+        <v>504</v>
       </c>
       <c r="P67" s="11" t="s">
-        <v>530</v>
+        <v>505</v>
       </c>
       <c r="Q67" s="19"/>
     </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A68" s="12" t="s">
-        <v>42</v>
+        <v>264</v>
       </c>
       <c r="B68" s="9">
-        <v>23573858468</v>
+        <v>13539917226</v>
       </c>
       <c r="C68" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>43</v>
+        <v>265</v>
       </c>
       <c r="E68" s="9" t="s">
-        <v>44</v>
+        <v>266</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="G68" s="18" t="s">
-        <v>534</v>
-      </c>
-      <c r="H68" s="2">
-        <v>70</v>
-      </c>
-      <c r="I68" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="G68" s="10" t="s">
+        <v>519</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="I68" s="4" t="s">
         <v>521</v>
       </c>
-      <c r="J68" s="2" t="s">
+      <c r="J68" s="4" t="s">
         <v>522</v>
       </c>
-      <c r="K68" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="L68" s="2" t="s">
+      <c r="K68" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="L68" s="4" t="s">
         <v>565</v>
       </c>
       <c r="M68" s="4" t="s">
         <v>579</v>
       </c>
-      <c r="N68" s="2">
+      <c r="N68" s="4">
         <v>3</v>
       </c>
       <c r="O68" s="11" t="s">
-        <v>532</v>
+        <v>517</v>
       </c>
       <c r="P68" s="11" t="s">
-        <v>533</v>
-      </c>
-      <c r="Q68" s="19" t="s">
-        <v>552</v>
-      </c>
+        <v>518</v>
+      </c>
+      <c r="Q68" s="19"/>
     </row>
     <row r="69" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A69" s="23" t="s">
-        <v>46</v>
+        <v>268</v>
       </c>
       <c r="B69" s="24">
-        <v>27406244206</v>
+        <v>18323004400</v>
       </c>
       <c r="C69" s="24" t="s">
         <v>6</v>
       </c>
       <c r="D69" s="24" t="s">
-        <v>47</v>
+        <v>269</v>
       </c>
       <c r="E69" s="24" t="s">
-        <v>48</v>
+        <v>270</v>
       </c>
       <c r="F69" s="24" t="s">
-        <v>49</v>
+        <v>271</v>
       </c>
       <c r="G69" s="25" t="s">
-        <v>537</v>
+        <v>524</v>
       </c>
       <c r="H69" s="7">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="I69" s="7" t="s">
         <v>521</v>
@@ -6447,7 +6445,7 @@
         <v>522</v>
       </c>
       <c r="K69" s="7" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="L69" s="7" t="s">
         <v>565</v>
@@ -6459,66 +6457,64 @@
         <v>3</v>
       </c>
       <c r="O69" s="26" t="s">
-        <v>535</v>
+        <v>507</v>
       </c>
       <c r="P69" s="26" t="s">
-        <v>536</v>
-      </c>
-      <c r="Q69" s="27" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.3">
+        <v>523</v>
+      </c>
+      <c r="Q69" s="27"/>
+    </row>
+    <row r="70" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A70" s="9" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="B70" s="9">
-        <v>13458064958</v>
+        <v>16388897646</v>
       </c>
       <c r="C70" s="9" t="s">
         <v>6</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="E70" s="9" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="F70" s="9" t="s">
-        <v>283</v>
-      </c>
-      <c r="G70" s="18" t="s">
-        <v>551</v>
-      </c>
-      <c r="H70" s="2">
-        <v>72</v>
-      </c>
-      <c r="I70" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="G70" s="10" t="s">
+        <v>527</v>
+      </c>
+      <c r="H70" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="I70" s="4" t="s">
         <v>521</v>
       </c>
-      <c r="J70" s="2" t="s">
+      <c r="J70" s="4" t="s">
         <v>522</v>
       </c>
-      <c r="K70" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="L70" s="2" t="s">
+      <c r="K70" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="L70" s="4" t="s">
         <v>565</v>
       </c>
       <c r="M70" s="4" t="s">
         <v>579</v>
       </c>
-      <c r="N70" s="2">
+      <c r="N70" s="4">
         <v>3</v>
       </c>
       <c r="O70" s="11" t="s">
-        <v>538</v>
+        <v>525</v>
       </c>
       <c r="P70" s="11" t="s">
-        <v>539</v>
+        <v>526</v>
       </c>
       <c r="Q70" s="9" t="s">
-        <v>554</v>
+        <v>580</v>
       </c>
     </row>
     <row r="71" spans="1:17" x14ac:dyDescent="0.3">

</xml_diff>